<commit_message>
feat: Adicionado funcao e regras para importacao no banco, finalizado necessario para processo
</commit_message>
<xml_diff>
--- a/03_-_arquivo_remessa_teste.xlsx
+++ b/03_-_arquivo_remessa_teste.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jodoarroyos\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DESENVOLVIMENTO\IMPORTACAO-IMPLANTACAO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C60CF481-D59E-43AD-925A-E074963C6736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321C6483-C775-4588-B8AE-D407998569DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26640" yWindow="2610" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Remessa" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Remessa!$A$1:$N$101</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -88,12 +91,6 @@
     <t>CTR1002</t>
   </si>
   <si>
-    <t>Maria Oliveira</t>
-  </si>
-  <si>
-    <t>maria@email.com</t>
-  </si>
-  <si>
     <t>31-02-2026</t>
   </si>
   <si>
@@ -115,10 +112,16 @@
     <t>CTR1004</t>
   </si>
   <si>
-    <t>Ana Costa</t>
+    <t>ana@email.com</t>
   </si>
   <si>
-    <t>ana@email.com</t>
+    <t>igor Oliveira</t>
+  </si>
+  <si>
+    <t>maria@email.com</t>
+  </si>
+  <si>
+    <t>Igor Henrique Alves</t>
   </si>
 </sst>
 </file>
@@ -128,10 +131,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -154,14 +165,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -527,10 +541,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -539,10 +553,10 @@
         <v>46062</v>
       </c>
       <c r="E2">
-        <v>402.29</v>
+        <v>325.47000000000003</v>
       </c>
       <c r="F2" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G2" t="s">
         <v>17</v>
@@ -551,7 +565,7 @@
         <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J2" s="1">
         <v>31187</v>
@@ -559,22 +573,22 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="1">
-        <v>46092</v>
+      <c r="D3" t="s">
+        <v>22</v>
       </c>
       <c r="E3">
-        <v>88.83</v>
+        <v>269.76</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
         <v>17</v>
@@ -583,7 +597,7 @@
         <v>18</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J3" s="1">
         <v>31187</v>
@@ -591,10 +605,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -603,10 +617,10 @@
         <v>46122</v>
       </c>
       <c r="E4">
-        <v>391.63</v>
+        <v>282.29000000000002</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
         <v>17</v>
@@ -615,7 +629,7 @@
         <v>18</v>
       </c>
       <c r="I4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J4" s="1">
         <v>31187</v>
@@ -623,10 +637,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -635,10 +649,10 @@
         <v>46152</v>
       </c>
       <c r="E5">
-        <v>73.790000000000006</v>
+        <v>282.75</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
         <v>17</v>
@@ -647,7 +661,7 @@
         <v>18</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J5" s="1">
         <v>31187</v>
@@ -655,10 +669,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -667,10 +681,10 @@
         <v>46182</v>
       </c>
       <c r="E6">
-        <v>276.54000000000002</v>
+        <v>233.26</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
         <v>17</v>
@@ -679,7 +693,7 @@
         <v>18</v>
       </c>
       <c r="I6" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J6" s="1">
         <v>31187</v>
@@ -687,10 +701,10 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -699,10 +713,10 @@
         <v>46212</v>
       </c>
       <c r="E7">
-        <v>110.65</v>
+        <v>322.86</v>
       </c>
       <c r="F7" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G7" t="s">
         <v>17</v>
@@ -711,7 +725,7 @@
         <v>18</v>
       </c>
       <c r="I7" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J7" s="1">
         <v>31187</v>
@@ -719,10 +733,10 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -731,10 +745,10 @@
         <v>46242</v>
       </c>
       <c r="E8">
-        <v>287.31</v>
+        <v>382.62</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
@@ -743,7 +757,7 @@
         <v>18</v>
       </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J8" s="1">
         <v>31187</v>
@@ -751,10 +765,10 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C9">
         <v>8</v>
@@ -763,10 +777,10 @@
         <v>46272</v>
       </c>
       <c r="E9">
-        <v>383</v>
+        <v>106.3</v>
       </c>
       <c r="F9" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
@@ -775,7 +789,7 @@
         <v>18</v>
       </c>
       <c r="I9" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J9" s="1">
         <v>31187</v>
@@ -783,10 +797,10 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -795,10 +809,10 @@
         <v>46302</v>
       </c>
       <c r="E10">
-        <v>220.21</v>
+        <v>439.45</v>
       </c>
       <c r="F10" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G10" t="s">
         <v>17</v>
@@ -807,7 +821,7 @@
         <v>18</v>
       </c>
       <c r="I10" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J10" s="1">
         <v>31187</v>
@@ -815,10 +829,10 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -827,10 +841,10 @@
         <v>46332</v>
       </c>
       <c r="E11">
-        <v>257.85000000000002</v>
+        <v>401.35</v>
       </c>
       <c r="F11" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G11" t="s">
         <v>17</v>
@@ -839,15 +853,18 @@
         <v>18</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J11" s="1">
         <v>31187</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C12">
         <v>11</v>
@@ -856,10 +873,10 @@
         <v>46362</v>
       </c>
       <c r="E12">
-        <v>50.3</v>
+        <v>464.31</v>
       </c>
       <c r="F12" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G12" t="s">
         <v>17</v>
@@ -868,7 +885,7 @@
         <v>18</v>
       </c>
       <c r="I12" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J12" s="1">
         <v>31187</v>
@@ -876,10 +893,10 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C13">
         <v>12</v>
@@ -888,10 +905,10 @@
         <v>46392</v>
       </c>
       <c r="E13">
-        <v>87.79</v>
+        <v>259.13</v>
       </c>
       <c r="F13" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G13" t="s">
         <v>17</v>
@@ -900,7 +917,7 @@
         <v>18</v>
       </c>
       <c r="I13" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J13" s="1">
         <v>31187</v>
@@ -908,10 +925,10 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C14">
         <v>13</v>
@@ -920,10 +937,10 @@
         <v>46422</v>
       </c>
       <c r="E14">
-        <v>261.58999999999997</v>
+        <v>137.30000000000001</v>
       </c>
       <c r="F14" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
@@ -932,7 +949,7 @@
         <v>18</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J14" s="1">
         <v>31187</v>
@@ -940,10 +957,10 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C15">
         <v>14</v>
@@ -952,10 +969,10 @@
         <v>46452</v>
       </c>
       <c r="E15">
-        <v>217.39</v>
+        <v>102.34</v>
       </c>
       <c r="F15" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G15" t="s">
         <v>17</v>
@@ -964,7 +981,7 @@
         <v>18</v>
       </c>
       <c r="I15" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J15" s="1">
         <v>31187</v>
@@ -972,10 +989,10 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C16">
         <v>15</v>
@@ -984,10 +1001,10 @@
         <v>46482</v>
       </c>
       <c r="E16">
-        <v>180.26</v>
+        <v>217.74</v>
       </c>
       <c r="F16" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G16" t="s">
         <v>17</v>
@@ -996,7 +1013,7 @@
         <v>18</v>
       </c>
       <c r="I16" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J16" s="1">
         <v>31187</v>
@@ -1004,10 +1021,10 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C17">
         <v>16</v>
@@ -1016,10 +1033,10 @@
         <v>46512</v>
       </c>
       <c r="E17">
-        <v>314.04000000000002</v>
+        <v>261.24</v>
       </c>
       <c r="F17" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G17" t="s">
         <v>17</v>
@@ -1028,7 +1045,7 @@
         <v>18</v>
       </c>
       <c r="I17" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J17" s="1">
         <v>31187</v>
@@ -1036,10 +1053,10 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C18">
         <v>17</v>
@@ -1048,10 +1065,10 @@
         <v>46542</v>
       </c>
       <c r="E18">
-        <v>136.37</v>
+        <v>206.59</v>
       </c>
       <c r="F18" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G18" t="s">
         <v>17</v>
@@ -1060,7 +1077,7 @@
         <v>18</v>
       </c>
       <c r="I18" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J18" s="1">
         <v>31187</v>
@@ -1068,10 +1085,10 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C19">
         <v>18</v>
@@ -1080,10 +1097,10 @@
         <v>46572</v>
       </c>
       <c r="E19">
-        <v>141.47</v>
+        <v>247.25</v>
       </c>
       <c r="F19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G19" t="s">
         <v>17</v>
@@ -1092,7 +1109,7 @@
         <v>18</v>
       </c>
       <c r="I19" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J19" s="1">
         <v>31187</v>
@@ -1100,10 +1117,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C20">
         <v>19</v>
@@ -1112,10 +1129,10 @@
         <v>46602</v>
       </c>
       <c r="E20">
-        <v>362.53</v>
+        <v>485.5</v>
       </c>
       <c r="F20" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G20" t="s">
         <v>17</v>
@@ -1124,7 +1141,7 @@
         <v>18</v>
       </c>
       <c r="I20" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J20" s="1">
         <v>31187</v>
@@ -1132,10 +1149,10 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C21">
         <v>20</v>
@@ -1144,10 +1161,10 @@
         <v>46632</v>
       </c>
       <c r="E21">
-        <v>388.2</v>
+        <v>309.33999999999997</v>
       </c>
       <c r="F21" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G21" t="s">
         <v>17</v>
@@ -1156,7 +1173,7 @@
         <v>18</v>
       </c>
       <c r="I21" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J21" s="1">
         <v>31187</v>
@@ -1164,10 +1181,10 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C22">
         <v>21</v>
@@ -1176,10 +1193,10 @@
         <v>46662</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>58.16</v>
       </c>
       <c r="F22" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G22" t="s">
         <v>17</v>
@@ -1188,7 +1205,7 @@
         <v>18</v>
       </c>
       <c r="I22" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J22" s="1">
         <v>31187</v>
@@ -1196,10 +1213,10 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C23">
         <v>22</v>
@@ -1208,10 +1225,10 @@
         <v>46692</v>
       </c>
       <c r="E23">
-        <v>324.7</v>
+        <v>125.44</v>
       </c>
       <c r="F23" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G23" t="s">
         <v>17</v>
@@ -1220,7 +1237,7 @@
         <v>18</v>
       </c>
       <c r="I23" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J23" s="1">
         <v>31187</v>
@@ -1228,10 +1245,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C24">
         <v>23</v>
@@ -1240,10 +1257,10 @@
         <v>46722</v>
       </c>
       <c r="E24">
-        <v>164.18</v>
+        <v>330.96</v>
       </c>
       <c r="F24" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G24" t="s">
         <v>17</v>
@@ -1252,7 +1269,7 @@
         <v>18</v>
       </c>
       <c r="I24" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J24" s="1">
         <v>31187</v>
@@ -1260,10 +1277,10 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C25">
         <v>24</v>
@@ -1272,10 +1289,10 @@
         <v>46752</v>
       </c>
       <c r="E25">
-        <v>103.72</v>
+        <v>214.94</v>
       </c>
       <c r="F25" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G25" t="s">
         <v>17</v>
@@ -1284,7 +1301,7 @@
         <v>18</v>
       </c>
       <c r="I25" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J25" s="1">
         <v>31187</v>
@@ -1292,10 +1309,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C26">
         <v>25</v>
@@ -1304,10 +1321,10 @@
         <v>46782</v>
       </c>
       <c r="E26">
-        <v>392.82</v>
+        <v>420</v>
       </c>
       <c r="F26" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G26" t="s">
         <v>17</v>
@@ -1316,7 +1333,7 @@
         <v>18</v>
       </c>
       <c r="I26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J26" s="1">
         <v>31187</v>
@@ -1324,10 +1341,10 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B27" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1336,10 +1353,10 @@
         <v>46062</v>
       </c>
       <c r="E27">
-        <v>270.81</v>
+        <v>74.14</v>
       </c>
       <c r="F27" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G27" t="s">
         <v>17</v>
@@ -1348,7 +1365,7 @@
         <v>18</v>
       </c>
       <c r="I27" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J27" s="1">
         <v>31187</v>
@@ -1356,10 +1373,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B28" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -1368,10 +1385,10 @@
         <v>46092</v>
       </c>
       <c r="E28">
-        <v>354.49</v>
+        <v>427.7</v>
       </c>
       <c r="F28" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G28" t="s">
         <v>17</v>
@@ -1380,7 +1397,7 @@
         <v>18</v>
       </c>
       <c r="I28" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J28" s="1">
         <v>31187</v>
@@ -1388,10 +1405,10 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B29" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C29">
         <v>3</v>
@@ -1400,10 +1417,10 @@
         <v>46122</v>
       </c>
       <c r="E29">
-        <v>261.52</v>
+        <v>66.94</v>
       </c>
       <c r="F29" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G29" t="s">
         <v>17</v>
@@ -1412,7 +1429,7 @@
         <v>18</v>
       </c>
       <c r="I29" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J29" s="1">
         <v>31187</v>
@@ -1420,10 +1437,10 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C30">
         <v>4</v>
@@ -1432,10 +1449,10 @@
         <v>46152</v>
       </c>
       <c r="E30">
-        <v>428.38</v>
+        <v>380.2</v>
       </c>
       <c r="F30" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G30" t="s">
         <v>17</v>
@@ -1444,7 +1461,7 @@
         <v>18</v>
       </c>
       <c r="I30" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J30" s="1">
         <v>31187</v>
@@ -1452,10 +1469,10 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C31">
         <v>5</v>
@@ -1464,10 +1481,10 @@
         <v>46182</v>
       </c>
       <c r="E31">
-        <v>320.37</v>
+        <v>494.48</v>
       </c>
       <c r="F31" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G31" t="s">
         <v>17</v>
@@ -1476,7 +1493,7 @@
         <v>18</v>
       </c>
       <c r="I31" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J31" s="1">
         <v>31187</v>
@@ -1484,10 +1501,10 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C32">
         <v>6</v>
@@ -1496,10 +1513,10 @@
         <v>46212</v>
       </c>
       <c r="E32">
-        <v>158.29</v>
+        <v>424.59</v>
       </c>
       <c r="F32" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G32" t="s">
         <v>17</v>
@@ -1508,7 +1525,7 @@
         <v>18</v>
       </c>
       <c r="I32" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J32" s="1">
         <v>31187</v>
@@ -1516,10 +1533,10 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B33" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C33">
         <v>7</v>
@@ -1528,10 +1545,10 @@
         <v>46242</v>
       </c>
       <c r="E33">
-        <v>273.72000000000003</v>
+        <v>289.45</v>
       </c>
       <c r="F33" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G33" t="s">
         <v>17</v>
@@ -1540,7 +1557,7 @@
         <v>18</v>
       </c>
       <c r="I33" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J33" s="1">
         <v>31187</v>
@@ -1548,10 +1565,10 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B34" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C34">
         <v>8</v>
@@ -1560,10 +1577,10 @@
         <v>46272</v>
       </c>
       <c r="E34">
-        <v>452.59</v>
+        <v>84.55</v>
       </c>
       <c r="F34" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G34" t="s">
         <v>17</v>
@@ -1572,7 +1589,7 @@
         <v>18</v>
       </c>
       <c r="I34" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J34" s="1">
         <v>31187</v>
@@ -1580,10 +1597,10 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C35">
         <v>9</v>
@@ -1592,10 +1609,10 @@
         <v>46302</v>
       </c>
       <c r="E35">
-        <v>487.92</v>
+        <v>0</v>
       </c>
       <c r="F35" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G35" t="s">
         <v>17</v>
@@ -1604,7 +1621,7 @@
         <v>18</v>
       </c>
       <c r="I35" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J35" s="1">
         <v>31187</v>
@@ -1612,10 +1629,10 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C36">
         <v>10</v>
@@ -1624,10 +1641,10 @@
         <v>46332</v>
       </c>
       <c r="E36">
-        <v>451.41</v>
+        <v>430.12</v>
       </c>
       <c r="F36" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G36" t="s">
         <v>17</v>
@@ -1636,7 +1653,7 @@
         <v>18</v>
       </c>
       <c r="I36" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J36" s="1">
         <v>31187</v>
@@ -1644,10 +1661,10 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C37">
         <v>11</v>
@@ -1656,10 +1673,10 @@
         <v>46362</v>
       </c>
       <c r="E37">
-        <v>83.56</v>
+        <v>494.54</v>
       </c>
       <c r="F37" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G37" t="s">
         <v>17</v>
@@ -1668,7 +1685,7 @@
         <v>18</v>
       </c>
       <c r="I37" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J37" s="1">
         <v>31187</v>
@@ -1676,10 +1693,10 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B38" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C38">
         <v>12</v>
@@ -1688,10 +1705,10 @@
         <v>46392</v>
       </c>
       <c r="E38">
-        <v>276.31</v>
+        <v>422.88</v>
       </c>
       <c r="F38" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G38" t="s">
         <v>17</v>
@@ -1700,15 +1717,18 @@
         <v>18</v>
       </c>
       <c r="I38" t="s">
+        <v>26</v>
+      </c>
+      <c r="J38" s="1">
+        <v>31187</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>23</v>
       </c>
-      <c r="J38" s="1">
-        <v>31187</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C39">
         <v>13</v>
@@ -1717,10 +1737,10 @@
         <v>46422</v>
       </c>
       <c r="E39">
-        <v>486.62</v>
+        <v>145.59</v>
       </c>
       <c r="F39" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G39" t="s">
         <v>17</v>
@@ -1729,7 +1749,7 @@
         <v>18</v>
       </c>
       <c r="I39" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J39" s="1">
         <v>31187</v>
@@ -1737,10 +1757,10 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B40" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C40">
         <v>14</v>
@@ -1749,10 +1769,10 @@
         <v>46452</v>
       </c>
       <c r="E40">
-        <v>200.89</v>
+        <v>342.33</v>
       </c>
       <c r="F40" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G40" t="s">
         <v>17</v>
@@ -1761,7 +1781,7 @@
         <v>18</v>
       </c>
       <c r="I40" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J40" s="1">
         <v>31187</v>
@@ -1769,10 +1789,10 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B41" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C41">
         <v>15</v>
@@ -1781,10 +1801,10 @@
         <v>46482</v>
       </c>
       <c r="E41">
-        <v>268.17</v>
+        <v>242.31</v>
       </c>
       <c r="F41" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G41" t="s">
         <v>17</v>
@@ -1793,7 +1813,7 @@
         <v>18</v>
       </c>
       <c r="I41" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J41" s="1">
         <v>31187</v>
@@ -1801,10 +1821,10 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B42" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C42">
         <v>16</v>
@@ -1813,10 +1833,10 @@
         <v>46512</v>
       </c>
       <c r="E42">
-        <v>375.72</v>
+        <v>364.2</v>
       </c>
       <c r="F42" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G42" t="s">
         <v>17</v>
@@ -1825,7 +1845,7 @@
         <v>18</v>
       </c>
       <c r="I42" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J42" s="1">
         <v>31187</v>
@@ -1833,10 +1853,10 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B43" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C43">
         <v>17</v>
@@ -1845,10 +1865,10 @@
         <v>46542</v>
       </c>
       <c r="E43">
-        <v>315.22000000000003</v>
+        <v>266.13</v>
       </c>
       <c r="F43" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G43" t="s">
         <v>17</v>
@@ -1857,7 +1877,7 @@
         <v>18</v>
       </c>
       <c r="I43" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J43" s="1">
         <v>31187</v>
@@ -1865,10 +1885,10 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C44">
         <v>18</v>
@@ -1877,10 +1897,10 @@
         <v>46572</v>
       </c>
       <c r="E44">
-        <v>243.17</v>
+        <v>480.81</v>
       </c>
       <c r="F44" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G44" t="s">
         <v>17</v>
@@ -1889,7 +1909,7 @@
         <v>18</v>
       </c>
       <c r="I44" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J44" s="1">
         <v>31187</v>
@@ -1897,10 +1917,10 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B45" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C45">
         <v>19</v>
@@ -1909,10 +1929,10 @@
         <v>46602</v>
       </c>
       <c r="E45">
-        <v>116.77</v>
+        <v>200.85</v>
       </c>
       <c r="F45" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G45" t="s">
         <v>17</v>
@@ -1921,7 +1941,7 @@
         <v>18</v>
       </c>
       <c r="I45" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J45" s="1">
         <v>31187</v>
@@ -1929,10 +1949,10 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B46" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C46">
         <v>20</v>
@@ -1941,10 +1961,10 @@
         <v>46632</v>
       </c>
       <c r="E46">
-        <v>498</v>
+        <v>499.49</v>
       </c>
       <c r="F46" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G46" t="s">
         <v>17</v>
@@ -1953,7 +1973,7 @@
         <v>18</v>
       </c>
       <c r="I46" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J46" s="1">
         <v>31187</v>
@@ -1961,22 +1981,22 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B47" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C47">
         <v>21</v>
       </c>
-      <c r="D47" t="s">
-        <v>24</v>
+      <c r="D47" s="1">
+        <v>46662</v>
       </c>
       <c r="E47">
-        <v>499.11</v>
+        <v>415.09</v>
       </c>
       <c r="F47" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G47" t="s">
         <v>17</v>
@@ -1985,7 +2005,7 @@
         <v>18</v>
       </c>
       <c r="I47" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J47" s="1">
         <v>31187</v>
@@ -1993,10 +2013,10 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B48" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C48">
         <v>22</v>
@@ -2005,10 +2025,10 @@
         <v>46692</v>
       </c>
       <c r="E48">
-        <v>164.73</v>
+        <v>294.85000000000002</v>
       </c>
       <c r="F48" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G48" t="s">
         <v>17</v>
@@ -2017,7 +2037,7 @@
         <v>18</v>
       </c>
       <c r="I48" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J48" s="1">
         <v>31187</v>
@@ -2025,10 +2045,10 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B49" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C49">
         <v>23</v>
@@ -2037,10 +2057,10 @@
         <v>46722</v>
       </c>
       <c r="E49">
-        <v>227.62</v>
+        <v>199.26</v>
       </c>
       <c r="F49" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G49" t="s">
         <v>17</v>
@@ -2049,7 +2069,7 @@
         <v>18</v>
       </c>
       <c r="I49" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J49" s="1">
         <v>31187</v>
@@ -2057,10 +2077,10 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B50" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C50">
         <v>24</v>
@@ -2069,10 +2089,10 @@
         <v>46752</v>
       </c>
       <c r="E50">
-        <v>80.23</v>
+        <v>494.72</v>
       </c>
       <c r="F50" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G50" t="s">
         <v>17</v>
@@ -2081,7 +2101,7 @@
         <v>18</v>
       </c>
       <c r="I50" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J50" s="1">
         <v>31187</v>
@@ -2089,10 +2109,10 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B51" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C51">
         <v>25</v>
@@ -2101,10 +2121,10 @@
         <v>46782</v>
       </c>
       <c r="E51">
-        <v>324.54000000000002</v>
+        <v>386.64</v>
       </c>
       <c r="F51" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G51" t="s">
         <v>17</v>
@@ -2113,7 +2133,7 @@
         <v>18</v>
       </c>
       <c r="I51" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J51" s="1">
         <v>31187</v>
@@ -2121,10 +2141,10 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B52" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2133,10 +2153,10 @@
         <v>46062</v>
       </c>
       <c r="E52">
-        <v>74.14</v>
+        <v>270.81</v>
       </c>
       <c r="F52" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G52" t="s">
         <v>17</v>
@@ -2144,8 +2164,8 @@
       <c r="H52" t="s">
         <v>18</v>
       </c>
-      <c r="I52" t="s">
-        <v>28</v>
+      <c r="I52" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J52" s="1">
         <v>31187</v>
@@ -2153,10 +2173,10 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B53" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C53">
         <v>2</v>
@@ -2165,10 +2185,10 @@
         <v>46092</v>
       </c>
       <c r="E53">
-        <v>427.7</v>
+        <v>354.49</v>
       </c>
       <c r="F53" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G53" t="s">
         <v>17</v>
@@ -2176,8 +2196,8 @@
       <c r="H53" t="s">
         <v>18</v>
       </c>
-      <c r="I53" t="s">
-        <v>28</v>
+      <c r="I53" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J53" s="1">
         <v>31187</v>
@@ -2185,10 +2205,10 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C54">
         <v>3</v>
@@ -2197,10 +2217,10 @@
         <v>46122</v>
       </c>
       <c r="E54">
-        <v>66.94</v>
+        <v>261.52</v>
       </c>
       <c r="F54" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G54" t="s">
         <v>17</v>
@@ -2208,8 +2228,8 @@
       <c r="H54" t="s">
         <v>18</v>
       </c>
-      <c r="I54" t="s">
-        <v>28</v>
+      <c r="I54" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J54" s="1">
         <v>31187</v>
@@ -2217,10 +2237,10 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C55">
         <v>4</v>
@@ -2229,10 +2249,10 @@
         <v>46152</v>
       </c>
       <c r="E55">
-        <v>380.2</v>
+        <v>428.38</v>
       </c>
       <c r="F55" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G55" t="s">
         <v>17</v>
@@ -2240,8 +2260,8 @@
       <c r="H55" t="s">
         <v>18</v>
       </c>
-      <c r="I55" t="s">
-        <v>28</v>
+      <c r="I55" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J55" s="1">
         <v>31187</v>
@@ -2249,10 +2269,10 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C56">
         <v>5</v>
@@ -2261,10 +2281,10 @@
         <v>46182</v>
       </c>
       <c r="E56">
-        <v>494.48</v>
+        <v>320.37</v>
       </c>
       <c r="F56" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G56" t="s">
         <v>17</v>
@@ -2272,8 +2292,8 @@
       <c r="H56" t="s">
         <v>18</v>
       </c>
-      <c r="I56" t="s">
-        <v>28</v>
+      <c r="I56" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J56" s="1">
         <v>31187</v>
@@ -2281,10 +2301,10 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C57">
         <v>6</v>
@@ -2293,10 +2313,10 @@
         <v>46212</v>
       </c>
       <c r="E57">
-        <v>424.59</v>
+        <v>158.29</v>
       </c>
       <c r="F57" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G57" t="s">
         <v>17</v>
@@ -2304,8 +2324,8 @@
       <c r="H57" t="s">
         <v>18</v>
       </c>
-      <c r="I57" t="s">
-        <v>28</v>
+      <c r="I57" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J57" s="1">
         <v>31187</v>
@@ -2313,10 +2333,10 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B58" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C58">
         <v>7</v>
@@ -2325,10 +2345,10 @@
         <v>46242</v>
       </c>
       <c r="E58">
-        <v>289.45</v>
+        <v>273.72000000000003</v>
       </c>
       <c r="F58" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G58" t="s">
         <v>17</v>
@@ -2336,8 +2356,8 @@
       <c r="H58" t="s">
         <v>18</v>
       </c>
-      <c r="I58" t="s">
-        <v>28</v>
+      <c r="I58" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J58" s="1">
         <v>31187</v>
@@ -2345,10 +2365,10 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C59">
         <v>8</v>
@@ -2357,10 +2377,10 @@
         <v>46272</v>
       </c>
       <c r="E59">
-        <v>84.55</v>
+        <v>452.59</v>
       </c>
       <c r="F59" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G59" t="s">
         <v>17</v>
@@ -2368,8 +2388,8 @@
       <c r="H59" t="s">
         <v>18</v>
       </c>
-      <c r="I59" t="s">
-        <v>28</v>
+      <c r="I59" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J59" s="1">
         <v>31187</v>
@@ -2377,10 +2397,10 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B60" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C60">
         <v>9</v>
@@ -2389,10 +2409,10 @@
         <v>46302</v>
       </c>
       <c r="E60">
-        <v>0</v>
+        <v>487.92</v>
       </c>
       <c r="F60" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G60" t="s">
         <v>17</v>
@@ -2400,8 +2420,8 @@
       <c r="H60" t="s">
         <v>18</v>
       </c>
-      <c r="I60" t="s">
-        <v>28</v>
+      <c r="I60" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J60" s="1">
         <v>31187</v>
@@ -2409,10 +2429,10 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C61">
         <v>10</v>
@@ -2421,10 +2441,10 @@
         <v>46332</v>
       </c>
       <c r="E61">
-        <v>430.12</v>
+        <v>451.41</v>
       </c>
       <c r="F61" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G61" t="s">
         <v>17</v>
@@ -2432,8 +2452,8 @@
       <c r="H61" t="s">
         <v>18</v>
       </c>
-      <c r="I61" t="s">
-        <v>28</v>
+      <c r="I61" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J61" s="1">
         <v>31187</v>
@@ -2441,10 +2461,10 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C62">
         <v>11</v>
@@ -2453,10 +2473,10 @@
         <v>46362</v>
       </c>
       <c r="E62">
-        <v>494.54</v>
+        <v>83.56</v>
       </c>
       <c r="F62" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G62" t="s">
         <v>17</v>
@@ -2464,8 +2484,8 @@
       <c r="H62" t="s">
         <v>18</v>
       </c>
-      <c r="I62" t="s">
-        <v>28</v>
+      <c r="I62" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J62" s="1">
         <v>31187</v>
@@ -2473,10 +2493,10 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B63" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C63">
         <v>12</v>
@@ -2485,10 +2505,10 @@
         <v>46392</v>
       </c>
       <c r="E63">
-        <v>422.88</v>
+        <v>276.31</v>
       </c>
       <c r="F63" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G63" t="s">
         <v>17</v>
@@ -2496,19 +2516,16 @@
       <c r="H63" t="s">
         <v>18</v>
       </c>
-      <c r="I63" t="s">
-        <v>28</v>
+      <c r="I63" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J63" s="1">
         <v>31187</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>25</v>
-      </c>
       <c r="B64" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C64">
         <v>13</v>
@@ -2517,10 +2534,10 @@
         <v>46422</v>
       </c>
       <c r="E64">
-        <v>145.59</v>
+        <v>486.62</v>
       </c>
       <c r="F64" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G64" t="s">
         <v>17</v>
@@ -2528,8 +2545,8 @@
       <c r="H64" t="s">
         <v>18</v>
       </c>
-      <c r="I64" t="s">
-        <v>28</v>
+      <c r="I64" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J64" s="1">
         <v>31187</v>
@@ -2537,10 +2554,10 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B65" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C65">
         <v>14</v>
@@ -2549,10 +2566,10 @@
         <v>46452</v>
       </c>
       <c r="E65">
-        <v>342.33</v>
+        <v>200.89</v>
       </c>
       <c r="F65" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G65" t="s">
         <v>17</v>
@@ -2560,8 +2577,8 @@
       <c r="H65" t="s">
         <v>18</v>
       </c>
-      <c r="I65" t="s">
-        <v>28</v>
+      <c r="I65" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J65" s="1">
         <v>31187</v>
@@ -2569,10 +2586,10 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B66" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C66">
         <v>15</v>
@@ -2581,10 +2598,10 @@
         <v>46482</v>
       </c>
       <c r="E66">
-        <v>242.31</v>
+        <v>268.17</v>
       </c>
       <c r="F66" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G66" t="s">
         <v>17</v>
@@ -2592,8 +2609,8 @@
       <c r="H66" t="s">
         <v>18</v>
       </c>
-      <c r="I66" t="s">
-        <v>28</v>
+      <c r="I66" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J66" s="1">
         <v>31187</v>
@@ -2601,10 +2618,10 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B67" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C67">
         <v>16</v>
@@ -2613,10 +2630,10 @@
         <v>46512</v>
       </c>
       <c r="E67">
-        <v>364.2</v>
+        <v>375.72</v>
       </c>
       <c r="F67" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G67" t="s">
         <v>17</v>
@@ -2624,8 +2641,8 @@
       <c r="H67" t="s">
         <v>18</v>
       </c>
-      <c r="I67" t="s">
-        <v>28</v>
+      <c r="I67" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J67" s="1">
         <v>31187</v>
@@ -2633,10 +2650,10 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B68" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C68">
         <v>17</v>
@@ -2645,10 +2662,10 @@
         <v>46542</v>
       </c>
       <c r="E68">
-        <v>266.13</v>
+        <v>315.22000000000003</v>
       </c>
       <c r="F68" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G68" t="s">
         <v>17</v>
@@ -2656,8 +2673,8 @@
       <c r="H68" t="s">
         <v>18</v>
       </c>
-      <c r="I68" t="s">
-        <v>28</v>
+      <c r="I68" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J68" s="1">
         <v>31187</v>
@@ -2665,10 +2682,10 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B69" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C69">
         <v>18</v>
@@ -2677,10 +2694,10 @@
         <v>46572</v>
       </c>
       <c r="E69">
-        <v>480.81</v>
+        <v>243.17</v>
       </c>
       <c r="F69" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G69" t="s">
         <v>17</v>
@@ -2688,8 +2705,8 @@
       <c r="H69" t="s">
         <v>18</v>
       </c>
-      <c r="I69" t="s">
-        <v>28</v>
+      <c r="I69" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J69" s="1">
         <v>31187</v>
@@ -2697,10 +2714,10 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B70" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C70">
         <v>19</v>
@@ -2709,10 +2726,10 @@
         <v>46602</v>
       </c>
       <c r="E70">
-        <v>200.85</v>
+        <v>116.77</v>
       </c>
       <c r="F70" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G70" t="s">
         <v>17</v>
@@ -2720,8 +2737,8 @@
       <c r="H70" t="s">
         <v>18</v>
       </c>
-      <c r="I70" t="s">
-        <v>28</v>
+      <c r="I70" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J70" s="1">
         <v>31187</v>
@@ -2729,10 +2746,10 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B71" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C71">
         <v>20</v>
@@ -2741,10 +2758,10 @@
         <v>46632</v>
       </c>
       <c r="E71">
-        <v>499.49</v>
+        <v>498</v>
       </c>
       <c r="F71" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G71" t="s">
         <v>17</v>
@@ -2752,8 +2769,8 @@
       <c r="H71" t="s">
         <v>18</v>
       </c>
-      <c r="I71" t="s">
-        <v>28</v>
+      <c r="I71" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J71" s="1">
         <v>31187</v>
@@ -2761,22 +2778,22 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C72">
         <v>21</v>
       </c>
-      <c r="D72" s="1">
-        <v>46662</v>
+      <c r="D72" t="s">
+        <v>22</v>
       </c>
       <c r="E72">
-        <v>415.09</v>
+        <v>499.11</v>
       </c>
       <c r="F72" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G72" t="s">
         <v>17</v>
@@ -2784,8 +2801,8 @@
       <c r="H72" t="s">
         <v>18</v>
       </c>
-      <c r="I72" t="s">
-        <v>28</v>
+      <c r="I72" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J72" s="1">
         <v>31187</v>
@@ -2793,10 +2810,10 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B73" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C73">
         <v>22</v>
@@ -2805,10 +2822,10 @@
         <v>46692</v>
       </c>
       <c r="E73">
-        <v>294.85000000000002</v>
+        <v>164.73</v>
       </c>
       <c r="F73" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G73" t="s">
         <v>17</v>
@@ -2816,8 +2833,8 @@
       <c r="H73" t="s">
         <v>18</v>
       </c>
-      <c r="I73" t="s">
-        <v>28</v>
+      <c r="I73" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J73" s="1">
         <v>31187</v>
@@ -2825,10 +2842,10 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B74" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C74">
         <v>23</v>
@@ -2837,10 +2854,10 @@
         <v>46722</v>
       </c>
       <c r="E74">
-        <v>199.26</v>
+        <v>227.62</v>
       </c>
       <c r="F74" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G74" t="s">
         <v>17</v>
@@ -2848,8 +2865,8 @@
       <c r="H74" t="s">
         <v>18</v>
       </c>
-      <c r="I74" t="s">
-        <v>28</v>
+      <c r="I74" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J74" s="1">
         <v>31187</v>
@@ -2857,10 +2874,10 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B75" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C75">
         <v>24</v>
@@ -2869,10 +2886,10 @@
         <v>46752</v>
       </c>
       <c r="E75">
-        <v>494.72</v>
+        <v>80.23</v>
       </c>
       <c r="F75" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G75" t="s">
         <v>17</v>
@@ -2880,8 +2897,8 @@
       <c r="H75" t="s">
         <v>18</v>
       </c>
-      <c r="I75" t="s">
-        <v>28</v>
+      <c r="I75" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J75" s="1">
         <v>31187</v>
@@ -2889,10 +2906,10 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B76" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C76">
         <v>25</v>
@@ -2901,10 +2918,10 @@
         <v>46782</v>
       </c>
       <c r="E76">
-        <v>386.64</v>
+        <v>324.54000000000002</v>
       </c>
       <c r="F76" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G76" t="s">
         <v>17</v>
@@ -2912,8 +2929,8 @@
       <c r="H76" t="s">
         <v>18</v>
       </c>
-      <c r="I76" t="s">
-        <v>28</v>
+      <c r="I76" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="J76" s="1">
         <v>31187</v>
@@ -2921,10 +2938,10 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -2933,10 +2950,10 @@
         <v>46062</v>
       </c>
       <c r="E77">
-        <v>325.47000000000003</v>
+        <v>402.29</v>
       </c>
       <c r="F77" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G77" t="s">
         <v>17</v>
@@ -2945,7 +2962,7 @@
         <v>18</v>
       </c>
       <c r="I77" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J77" s="1">
         <v>31187</v>
@@ -2953,22 +2970,22 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C78">
         <v>2</v>
       </c>
-      <c r="D78" t="s">
-        <v>24</v>
+      <c r="D78" s="1">
+        <v>46092</v>
       </c>
       <c r="E78">
-        <v>269.76</v>
+        <v>88.83</v>
       </c>
       <c r="F78" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G78" t="s">
         <v>17</v>
@@ -2977,7 +2994,7 @@
         <v>18</v>
       </c>
       <c r="I78" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J78" s="1">
         <v>31187</v>
@@ -2985,10 +3002,10 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C79">
         <v>3</v>
@@ -2997,10 +3014,10 @@
         <v>46122</v>
       </c>
       <c r="E79">
-        <v>282.29000000000002</v>
+        <v>391.63</v>
       </c>
       <c r="F79" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G79" t="s">
         <v>17</v>
@@ -3009,7 +3026,7 @@
         <v>18</v>
       </c>
       <c r="I79" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J79" s="1">
         <v>31187</v>
@@ -3017,10 +3034,10 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C80">
         <v>4</v>
@@ -3029,10 +3046,10 @@
         <v>46152</v>
       </c>
       <c r="E80">
-        <v>282.75</v>
+        <v>73.790000000000006</v>
       </c>
       <c r="F80" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G80" t="s">
         <v>17</v>
@@ -3041,7 +3058,7 @@
         <v>18</v>
       </c>
       <c r="I80" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J80" s="1">
         <v>31187</v>
@@ -3049,10 +3066,10 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B81" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C81">
         <v>5</v>
@@ -3061,10 +3078,10 @@
         <v>46182</v>
       </c>
       <c r="E81">
-        <v>233.26</v>
+        <v>276.54000000000002</v>
       </c>
       <c r="F81" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G81" t="s">
         <v>17</v>
@@ -3073,7 +3090,7 @@
         <v>18</v>
       </c>
       <c r="I81" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J81" s="1">
         <v>31187</v>
@@ -3081,10 +3098,10 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C82">
         <v>6</v>
@@ -3093,10 +3110,10 @@
         <v>46212</v>
       </c>
       <c r="E82">
-        <v>322.86</v>
+        <v>110.65</v>
       </c>
       <c r="F82" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G82" t="s">
         <v>17</v>
@@ -3105,7 +3122,7 @@
         <v>18</v>
       </c>
       <c r="I82" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J82" s="1">
         <v>31187</v>
@@ -3113,10 +3130,10 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B83" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C83">
         <v>7</v>
@@ -3125,10 +3142,10 @@
         <v>46242</v>
       </c>
       <c r="E83">
-        <v>382.62</v>
+        <v>287.31</v>
       </c>
       <c r="F83" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G83" t="s">
         <v>17</v>
@@ -3137,7 +3154,7 @@
         <v>18</v>
       </c>
       <c r="I83" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J83" s="1">
         <v>31187</v>
@@ -3145,10 +3162,10 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C84">
         <v>8</v>
@@ -3157,10 +3174,10 @@
         <v>46272</v>
       </c>
       <c r="E84">
-        <v>106.3</v>
+        <v>383</v>
       </c>
       <c r="F84" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G84" t="s">
         <v>17</v>
@@ -3169,7 +3186,7 @@
         <v>18</v>
       </c>
       <c r="I84" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J84" s="1">
         <v>31187</v>
@@ -3177,10 +3194,10 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C85">
         <v>9</v>
@@ -3189,10 +3206,10 @@
         <v>46302</v>
       </c>
       <c r="E85">
-        <v>439.45</v>
+        <v>220.21</v>
       </c>
       <c r="F85" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G85" t="s">
         <v>17</v>
@@ -3201,7 +3218,7 @@
         <v>18</v>
       </c>
       <c r="I85" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J85" s="1">
         <v>31187</v>
@@ -3209,10 +3226,10 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C86">
         <v>10</v>
@@ -3221,10 +3238,10 @@
         <v>46332</v>
       </c>
       <c r="E86">
-        <v>401.35</v>
+        <v>257.85000000000002</v>
       </c>
       <c r="F86" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G86" t="s">
         <v>17</v>
@@ -3233,18 +3250,15 @@
         <v>18</v>
       </c>
       <c r="I86" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J86" s="1">
         <v>31187</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>29</v>
-      </c>
       <c r="B87" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C87">
         <v>11</v>
@@ -3253,10 +3267,10 @@
         <v>46362</v>
       </c>
       <c r="E87">
-        <v>464.31</v>
+        <v>50.3</v>
       </c>
       <c r="F87" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G87" t="s">
         <v>17</v>
@@ -3265,7 +3279,7 @@
         <v>18</v>
       </c>
       <c r="I87" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J87" s="1">
         <v>31187</v>
@@ -3273,10 +3287,10 @@
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C88">
         <v>12</v>
@@ -3285,10 +3299,10 @@
         <v>46392</v>
       </c>
       <c r="E88">
-        <v>259.13</v>
+        <v>87.79</v>
       </c>
       <c r="F88" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G88" t="s">
         <v>17</v>
@@ -3297,7 +3311,7 @@
         <v>18</v>
       </c>
       <c r="I88" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J88" s="1">
         <v>31187</v>
@@ -3305,10 +3319,10 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B89" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C89">
         <v>13</v>
@@ -3317,10 +3331,10 @@
         <v>46422</v>
       </c>
       <c r="E89">
-        <v>137.30000000000001</v>
+        <v>261.58999999999997</v>
       </c>
       <c r="F89" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G89" t="s">
         <v>17</v>
@@ -3329,7 +3343,7 @@
         <v>18</v>
       </c>
       <c r="I89" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J89" s="1">
         <v>31187</v>
@@ -3337,10 +3351,10 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B90" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C90">
         <v>14</v>
@@ -3349,10 +3363,10 @@
         <v>46452</v>
       </c>
       <c r="E90">
-        <v>102.34</v>
+        <v>217.39</v>
       </c>
       <c r="F90" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G90" t="s">
         <v>17</v>
@@ -3361,7 +3375,7 @@
         <v>18</v>
       </c>
       <c r="I90" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J90" s="1">
         <v>31187</v>
@@ -3369,10 +3383,10 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B91" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C91">
         <v>15</v>
@@ -3381,10 +3395,10 @@
         <v>46482</v>
       </c>
       <c r="E91">
-        <v>217.74</v>
+        <v>180.26</v>
       </c>
       <c r="F91" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G91" t="s">
         <v>17</v>
@@ -3393,7 +3407,7 @@
         <v>18</v>
       </c>
       <c r="I91" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J91" s="1">
         <v>31187</v>
@@ -3401,10 +3415,10 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B92" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C92">
         <v>16</v>
@@ -3413,10 +3427,10 @@
         <v>46512</v>
       </c>
       <c r="E92">
-        <v>261.24</v>
+        <v>314.04000000000002</v>
       </c>
       <c r="F92" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G92" t="s">
         <v>17</v>
@@ -3425,7 +3439,7 @@
         <v>18</v>
       </c>
       <c r="I92" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J92" s="1">
         <v>31187</v>
@@ -3433,10 +3447,10 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B93" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C93">
         <v>17</v>
@@ -3445,10 +3459,10 @@
         <v>46542</v>
       </c>
       <c r="E93">
-        <v>206.59</v>
+        <v>136.37</v>
       </c>
       <c r="F93" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G93" t="s">
         <v>17</v>
@@ -3457,7 +3471,7 @@
         <v>18</v>
       </c>
       <c r="I93" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J93" s="1">
         <v>31187</v>
@@ -3465,10 +3479,10 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B94" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C94">
         <v>18</v>
@@ -3477,10 +3491,10 @@
         <v>46572</v>
       </c>
       <c r="E94">
-        <v>247.25</v>
+        <v>141.47</v>
       </c>
       <c r="F94" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G94" t="s">
         <v>17</v>
@@ -3489,7 +3503,7 @@
         <v>18</v>
       </c>
       <c r="I94" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J94" s="1">
         <v>31187</v>
@@ -3497,10 +3511,10 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B95" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C95">
         <v>19</v>
@@ -3509,10 +3523,10 @@
         <v>46602</v>
       </c>
       <c r="E95">
-        <v>485.5</v>
+        <v>362.53</v>
       </c>
       <c r="F95" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G95" t="s">
         <v>17</v>
@@ -3521,7 +3535,7 @@
         <v>18</v>
       </c>
       <c r="I95" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J95" s="1">
         <v>31187</v>
@@ -3529,10 +3543,10 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B96" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C96">
         <v>20</v>
@@ -3541,10 +3555,10 @@
         <v>46632</v>
       </c>
       <c r="E96">
-        <v>309.33999999999997</v>
+        <v>388.2</v>
       </c>
       <c r="F96" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G96" t="s">
         <v>17</v>
@@ -3553,7 +3567,7 @@
         <v>18</v>
       </c>
       <c r="I96" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J96" s="1">
         <v>31187</v>
@@ -3561,10 +3575,10 @@
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B97" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C97">
         <v>21</v>
@@ -3573,10 +3587,10 @@
         <v>46662</v>
       </c>
       <c r="E97">
-        <v>58.16</v>
+        <v>0</v>
       </c>
       <c r="F97" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G97" t="s">
         <v>17</v>
@@ -3585,7 +3599,7 @@
         <v>18</v>
       </c>
       <c r="I97" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J97" s="1">
         <v>31187</v>
@@ -3593,10 +3607,10 @@
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B98" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C98">
         <v>22</v>
@@ -3605,10 +3619,10 @@
         <v>46692</v>
       </c>
       <c r="E98">
-        <v>125.44</v>
+        <v>324.7</v>
       </c>
       <c r="F98" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G98" t="s">
         <v>17</v>
@@ -3617,7 +3631,7 @@
         <v>18</v>
       </c>
       <c r="I98" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J98" s="1">
         <v>31187</v>
@@ -3625,10 +3639,10 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B99" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C99">
         <v>23</v>
@@ -3637,10 +3651,10 @@
         <v>46722</v>
       </c>
       <c r="E99">
-        <v>330.96</v>
+        <v>164.18</v>
       </c>
       <c r="F99" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G99" t="s">
         <v>17</v>
@@ -3649,7 +3663,7 @@
         <v>18</v>
       </c>
       <c r="I99" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J99" s="1">
         <v>31187</v>
@@ -3657,10 +3671,10 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B100" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C100">
         <v>24</v>
@@ -3669,10 +3683,10 @@
         <v>46752</v>
       </c>
       <c r="E100">
-        <v>214.94</v>
+        <v>103.72</v>
       </c>
       <c r="F100" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G100" t="s">
         <v>17</v>
@@ -3681,7 +3695,7 @@
         <v>18</v>
       </c>
       <c r="I100" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J100" s="1">
         <v>31187</v>
@@ -3689,10 +3703,10 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B101" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C101">
         <v>25</v>
@@ -3701,10 +3715,10 @@
         <v>46782</v>
       </c>
       <c r="E101">
-        <v>420</v>
+        <v>392.82</v>
       </c>
       <c r="F101" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G101" t="s">
         <v>17</v>
@@ -3713,7 +3727,7 @@
         <v>18</v>
       </c>
       <c r="I101" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J101" s="1">
         <v>31187</v>

</xml_diff>